<commit_message>
Add official Anthropic prices next to OpenRouter prices
Parse the Anthropic pricing docs (Markdown version) for standard and
batch prices, compare them with OpenRouter, and add Anthropic models
missing from OpenRouter as new rows. The official-price columns are now
provider-neutral so OpenAI and Anthropic share them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmrknBAh1G6gZXqySqNkyo
</commit_message>
<xml_diff>
--- a/openrouter_prices.xlsx
+++ b/openrouter_prices.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Cohere" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All'!$A$1:$T$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All'!$A$1:$T$205</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OpenAI'!$A$1:$T$147</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Anthropic'!$A$1:$L$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Anthropic'!$A$1:$T$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DeepSeek'!$A$1:$L$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cohere'!$A$1:$L$7</definedName>
   </definedNames>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T199"/>
+  <dimension ref="A1:T210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -555,32 +555,32 @@
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI model</t>
+          <t>Official model</t>
         </is>
       </c>
       <c r="N1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI tier</t>
+          <t>Official tier</t>
         </is>
       </c>
       <c r="O1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Input $/1M</t>
+          <t>Official Input $/1M</t>
         </is>
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Cached input $/1M</t>
+          <t>Official Cached input $/1M</t>
         </is>
       </c>
       <c r="Q1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Cache write $/1M</t>
+          <t>Official Cache write $/1M</t>
         </is>
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Output $/1M</t>
+          <t>Official Output $/1M</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="T1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI note</t>
+          <t>Official note</t>
         </is>
       </c>
     </row>
@@ -6246,10 +6246,38 @@
       <c r="L102" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O102" s="4" t="n"/>
-      <c r="P102" s="4" t="n"/>
-      <c r="Q102" s="4" t="n"/>
-      <c r="R102" s="4" t="n"/>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>claude-fable-5</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O102" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P102" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q102" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R102" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S102" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>1h cache write: $20</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6288,10 +6316,38 @@
       <c r="L103" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O103" s="4" t="n"/>
-      <c r="P103" s="4" t="n"/>
-      <c r="Q103" s="4" t="n"/>
-      <c r="R103" s="4" t="n"/>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>claude-fable-5.1</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O103" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P103" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q103" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R103" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S103" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>1h cache write: $20</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6330,10 +6386,29 @@
       <c r="L104" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O104" s="4" t="n"/>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>claude-fable-5.1</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O104" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="P104" s="4" t="n"/>
       <c r="Q104" s="4" t="n"/>
-      <c r="R104" s="4" t="n"/>
+      <c r="R104" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S104" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6372,10 +6447,29 @@
       <c r="L105" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O105" s="4" t="n"/>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>claude-fable-5</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O105" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="P105" s="4" t="n"/>
       <c r="Q105" s="4" t="n"/>
-      <c r="R105" s="4" t="n"/>
+      <c r="R105" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S105" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6414,10 +6508,38 @@
       <c r="L106" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O106" s="4" t="n"/>
-      <c r="P106" s="4" t="n"/>
-      <c r="Q106" s="4" t="n"/>
-      <c r="R106" s="4" t="n"/>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>claude-haiku-4.5</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O106" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P106" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q106" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="R106" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S106" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>1h cache write: $2</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6456,10 +6578,29 @@
       <c r="L107" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O107" s="4" t="n"/>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>claude-haiku-4.5</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O107" s="4" t="n">
+        <v>0.5</v>
+      </c>
       <c r="P107" s="4" t="n"/>
       <c r="Q107" s="4" t="n"/>
-      <c r="R107" s="4" t="n"/>
+      <c r="R107" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S107" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6498,10 +6639,38 @@
       <c r="L108" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O108" s="4" t="n"/>
-      <c r="P108" s="4" t="n"/>
-      <c r="Q108" s="4" t="n"/>
-      <c r="R108" s="4" t="n"/>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>claude-opus-4.1</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O108" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P108" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q108" s="4" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="R108" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="S108" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>1h cache write: $30; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6540,10 +6709,34 @@
       <c r="L109" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O109" s="4" t="n"/>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>claude-opus-4.1</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O109" s="4" t="n">
+        <v>7.5</v>
+      </c>
       <c r="P109" s="4" t="n"/>
       <c r="Q109" s="4" t="n"/>
-      <c r="R109" s="4" t="n"/>
+      <c r="R109" s="4" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="S109" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6582,10 +6775,38 @@
       <c r="L110" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O110" s="4" t="n"/>
-      <c r="P110" s="4" t="n"/>
-      <c r="Q110" s="4" t="n"/>
-      <c r="R110" s="4" t="n"/>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>claude-opus-4.5</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O110" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P110" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q110" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R110" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S110" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6624,10 +6845,29 @@
       <c r="L111" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O111" s="4" t="n"/>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>claude-opus-4.5</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O111" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P111" s="4" t="n"/>
       <c r="Q111" s="4" t="n"/>
-      <c r="R111" s="4" t="n"/>
+      <c r="R111" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S111" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6666,10 +6906,38 @@
       <c r="L112" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O112" s="4" t="n"/>
-      <c r="P112" s="4" t="n"/>
-      <c r="Q112" s="4" t="n"/>
-      <c r="R112" s="4" t="n"/>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>claude-opus-4.6</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O112" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P112" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q112" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R112" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S112" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6708,10 +6976,29 @@
       <c r="L113" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O113" s="4" t="n"/>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>claude-opus-4.6</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O113" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P113" s="4" t="n"/>
       <c r="Q113" s="4" t="n"/>
-      <c r="R113" s="4" t="n"/>
+      <c r="R113" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S113" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6750,10 +7037,38 @@
       <c r="L114" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O114" s="4" t="n"/>
-      <c r="P114" s="4" t="n"/>
-      <c r="Q114" s="4" t="n"/>
-      <c r="R114" s="4" t="n"/>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>claude-opus-4.7</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O114" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P114" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q114" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R114" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S114" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6792,10 +7107,29 @@
       <c r="L115" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O115" s="4" t="n"/>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>claude-opus-4.7</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O115" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P115" s="4" t="n"/>
       <c r="Q115" s="4" t="n"/>
-      <c r="R115" s="4" t="n"/>
+      <c r="R115" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S115" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6834,10 +7168,38 @@
       <c r="L116" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O116" s="4" t="n"/>
-      <c r="P116" s="4" t="n"/>
-      <c r="Q116" s="4" t="n"/>
-      <c r="R116" s="4" t="n"/>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>claude-opus-4.8</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O116" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P116" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q116" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R116" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S116" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6876,10 +7238,29 @@
       <c r="L117" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O117" s="4" t="n"/>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>claude-opus-4.8</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O117" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P117" s="4" t="n"/>
       <c r="Q117" s="4" t="n"/>
-      <c r="R117" s="4" t="n"/>
+      <c r="R117" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S117" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6918,10 +7299,38 @@
       <c r="L118" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O118" s="4" t="n"/>
-      <c r="P118" s="4" t="n"/>
-      <c r="Q118" s="4" t="n"/>
-      <c r="R118" s="4" t="n"/>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>claude-opus-5</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O118" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P118" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q118" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R118" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S118" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6960,10 +7369,38 @@
       <c r="L119" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O119" s="4" t="n"/>
-      <c r="P119" s="4" t="n"/>
-      <c r="Q119" s="4" t="n"/>
-      <c r="R119" s="4" t="n"/>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>claude-opus-5.5</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O119" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P119" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q119" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R119" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S119" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>1h cache write: $8</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7002,10 +7439,29 @@
       <c r="L120" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O120" s="4" t="n"/>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>claude-opus-5.5</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O120" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P120" s="4" t="n"/>
       <c r="Q120" s="4" t="n"/>
-      <c r="R120" s="4" t="n"/>
+      <c r="R120" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S120" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7044,10 +7500,29 @@
       <c r="L121" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O121" s="4" t="n"/>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>claude-opus-5</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O121" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P121" s="4" t="n"/>
       <c r="Q121" s="4" t="n"/>
-      <c r="R121" s="4" t="n"/>
+      <c r="R121" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S121" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7086,10 +7561,38 @@
       <c r="L122" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O122" s="4" t="n"/>
-      <c r="P122" s="4" t="n"/>
-      <c r="Q122" s="4" t="n"/>
-      <c r="R122" s="4" t="n"/>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O122" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P122" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q122" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R122" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S122" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>1h cache write: $6; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7128,10 +7631,38 @@
       <c r="L123" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O123" s="4" t="n"/>
-      <c r="P123" s="4" t="n"/>
-      <c r="Q123" s="4" t="n"/>
-      <c r="R123" s="4" t="n"/>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.5</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O123" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P123" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q123" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R123" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S123" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>1h cache write: $6</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7170,10 +7701,29 @@
       <c r="L124" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O124" s="4" t="n"/>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.5</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O124" s="4" t="n">
+        <v>1.5</v>
+      </c>
       <c r="P124" s="4" t="n"/>
       <c r="Q124" s="4" t="n"/>
-      <c r="R124" s="4" t="n"/>
+      <c r="R124" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S124" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7212,10 +7762,38 @@
       <c r="L125" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O125" s="4" t="n"/>
-      <c r="P125" s="4" t="n"/>
-      <c r="Q125" s="4" t="n"/>
-      <c r="R125" s="4" t="n"/>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.6</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O125" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P125" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q125" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R125" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S125" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>1h cache write: $6</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7254,10 +7832,29 @@
       <c r="L126" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O126" s="4" t="n"/>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.6</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O126" s="4" t="n">
+        <v>1.5</v>
+      </c>
       <c r="P126" s="4" t="n"/>
       <c r="Q126" s="4" t="n"/>
-      <c r="R126" s="4" t="n"/>
+      <c r="R126" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S126" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7296,10 +7893,38 @@
       <c r="L127" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O127" s="4" t="n"/>
-      <c r="P127" s="4" t="n"/>
-      <c r="Q127" s="4" t="n"/>
-      <c r="R127" s="4" t="n"/>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O127" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P127" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q127" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="R127" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S127" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>1h cache write: $4</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7338,10 +7963,29 @@
       <c r="L128" s="4" t="n">
         <v>0.01</v>
       </c>
-      <c r="O128" s="4" t="n"/>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O128" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P128" s="4" t="n"/>
       <c r="Q128" s="4" t="n"/>
-      <c r="R128" s="4" t="n"/>
+      <c r="R128" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S128" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10219,22 +10863,466 @@
       </c>
       <c r="T196" s="7" t="n"/>
     </row>
+    <row r="197">
+      <c r="A197" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B197" s="7" t="n"/>
+      <c r="C197" s="7" t="n"/>
+      <c r="D197" s="8" t="n"/>
+      <c r="E197" s="9" t="n"/>
+      <c r="F197" s="9" t="n"/>
+      <c r="G197" s="9" t="n"/>
+      <c r="H197" s="9" t="n"/>
+      <c r="I197" s="9" t="n"/>
+      <c r="J197" s="9" t="n"/>
+      <c r="K197" s="9" t="n"/>
+      <c r="L197" s="9" t="n"/>
+      <c r="M197" s="7" t="inlineStr">
+        <is>
+          <t>claude-haiku-3.5</t>
+        </is>
+      </c>
+      <c r="N197" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O197" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P197" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q197" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R197" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S197" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T197" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $1.6; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
+    </row>
     <row r="198">
-      <c r="A198" t="inlineStr">
+      <c r="A198" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B198" s="7" t="n"/>
+      <c r="C198" s="7" t="n"/>
+      <c r="D198" s="8" t="n"/>
+      <c r="E198" s="9" t="n"/>
+      <c r="F198" s="9" t="n"/>
+      <c r="G198" s="9" t="n"/>
+      <c r="H198" s="9" t="n"/>
+      <c r="I198" s="9" t="n"/>
+      <c r="J198" s="9" t="n"/>
+      <c r="K198" s="9" t="n"/>
+      <c r="L198" s="9" t="n"/>
+      <c r="M198" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5</t>
+        </is>
+      </c>
+      <c r="N198" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O198" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P198" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q198" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R198" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="S198" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T198" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $20; limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B199" s="7" t="n"/>
+      <c r="C199" s="7" t="n"/>
+      <c r="D199" s="8" t="n"/>
+      <c r="E199" s="9" t="n"/>
+      <c r="F199" s="9" t="n"/>
+      <c r="G199" s="9" t="n"/>
+      <c r="H199" s="9" t="n"/>
+      <c r="I199" s="9" t="n"/>
+      <c r="J199" s="9" t="n"/>
+      <c r="K199" s="9" t="n"/>
+      <c r="L199" s="9" t="n"/>
+      <c r="M199" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5.1</t>
+        </is>
+      </c>
+      <c r="N199" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O199" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P199" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q199" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R199" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="S199" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T199" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $20; limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B200" s="7" t="n"/>
+      <c r="C200" s="7" t="n"/>
+      <c r="D200" s="8" t="n"/>
+      <c r="E200" s="9" t="n"/>
+      <c r="F200" s="9" t="n"/>
+      <c r="G200" s="9" t="n"/>
+      <c r="H200" s="9" t="n"/>
+      <c r="I200" s="9" t="n"/>
+      <c r="J200" s="9" t="n"/>
+      <c r="K200" s="9" t="n"/>
+      <c r="L200" s="9" t="n"/>
+      <c r="M200" s="7" t="inlineStr">
+        <is>
+          <t>claude-opus-4</t>
+        </is>
+      </c>
+      <c r="N200" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O200" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="P200" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q200" s="9" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="R200" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="S200" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T200" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $30; retired, except on Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B201" s="7" t="n"/>
+      <c r="C201" s="7" t="n"/>
+      <c r="D201" s="8" t="n"/>
+      <c r="E201" s="9" t="n"/>
+      <c r="F201" s="9" t="n"/>
+      <c r="G201" s="9" t="n"/>
+      <c r="H201" s="9" t="n"/>
+      <c r="I201" s="9" t="n"/>
+      <c r="J201" s="9" t="n"/>
+      <c r="K201" s="9" t="n"/>
+      <c r="L201" s="9" t="n"/>
+      <c r="M201" s="7" t="inlineStr">
+        <is>
+          <t>claude-haiku-3.5</t>
+        </is>
+      </c>
+      <c r="N201" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O201" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P201" s="9" t="n"/>
+      <c r="Q201" s="9" t="n"/>
+      <c r="R201" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S201" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T201" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B202" s="7" t="n"/>
+      <c r="C202" s="7" t="n"/>
+      <c r="D202" s="8" t="n"/>
+      <c r="E202" s="9" t="n"/>
+      <c r="F202" s="9" t="n"/>
+      <c r="G202" s="9" t="n"/>
+      <c r="H202" s="9" t="n"/>
+      <c r="I202" s="9" t="n"/>
+      <c r="J202" s="9" t="n"/>
+      <c r="K202" s="9" t="n"/>
+      <c r="L202" s="9" t="n"/>
+      <c r="M202" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5</t>
+        </is>
+      </c>
+      <c r="N202" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O202" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P202" s="9" t="n"/>
+      <c r="Q202" s="9" t="n"/>
+      <c r="R202" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="S202" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T202" s="7" t="inlineStr">
+        <is>
+          <t>limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B203" s="7" t="n"/>
+      <c r="C203" s="7" t="n"/>
+      <c r="D203" s="8" t="n"/>
+      <c r="E203" s="9" t="n"/>
+      <c r="F203" s="9" t="n"/>
+      <c r="G203" s="9" t="n"/>
+      <c r="H203" s="9" t="n"/>
+      <c r="I203" s="9" t="n"/>
+      <c r="J203" s="9" t="n"/>
+      <c r="K203" s="9" t="n"/>
+      <c r="L203" s="9" t="n"/>
+      <c r="M203" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5.1</t>
+        </is>
+      </c>
+      <c r="N203" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O203" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P203" s="9" t="n"/>
+      <c r="Q203" s="9" t="n"/>
+      <c r="R203" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="S203" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T203" s="7" t="inlineStr">
+        <is>
+          <t>limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B204" s="7" t="n"/>
+      <c r="C204" s="7" t="n"/>
+      <c r="D204" s="8" t="n"/>
+      <c r="E204" s="9" t="n"/>
+      <c r="F204" s="9" t="n"/>
+      <c r="G204" s="9" t="n"/>
+      <c r="H204" s="9" t="n"/>
+      <c r="I204" s="9" t="n"/>
+      <c r="J204" s="9" t="n"/>
+      <c r="K204" s="9" t="n"/>
+      <c r="L204" s="9" t="n"/>
+      <c r="M204" s="7" t="inlineStr">
+        <is>
+          <t>claude-opus-4</t>
+        </is>
+      </c>
+      <c r="N204" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O204" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P204" s="9" t="n"/>
+      <c r="Q204" s="9" t="n"/>
+      <c r="R204" s="9" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="S204" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T204" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B205" s="7" t="n"/>
+      <c r="C205" s="7" t="n"/>
+      <c r="D205" s="8" t="n"/>
+      <c r="E205" s="9" t="n"/>
+      <c r="F205" s="9" t="n"/>
+      <c r="G205" s="9" t="n"/>
+      <c r="H205" s="9" t="n"/>
+      <c r="I205" s="9" t="n"/>
+      <c r="J205" s="9" t="n"/>
+      <c r="K205" s="9" t="n"/>
+      <c r="L205" s="9" t="n"/>
+      <c r="M205" s="7" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4</t>
+        </is>
+      </c>
+      <c r="N205" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O205" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P205" s="9" t="n"/>
+      <c r="Q205" s="9" t="n"/>
+      <c r="R205" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S205" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T205" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
         <is>
           <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
         </is>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>Green columns: official OpenAI prices from https://developers.openai.com/api/docs/pricing (Standard tier; Batch tier for ':batch' models). Yellow rows: models OpenRouter does not list.</t>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Green columns (OpenAI): official prices from https://developers.openai.com/api/docs/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Green columns (Anthropic): official prices from https://platform.claude.com/docs/en/about-claude/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T196"/>
+  <autoFilter ref="A1:T205"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10245,7 +11333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T150"/>
+  <dimension ref="A1:T151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10333,32 +11421,32 @@
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI model</t>
+          <t>Official model</t>
         </is>
       </c>
       <c r="N1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI tier</t>
+          <t>Official tier</t>
         </is>
       </c>
       <c r="O1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Input $/1M</t>
+          <t>Official Input $/1M</t>
         </is>
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Cached input $/1M</t>
+          <t>Official Cached input $/1M</t>
         </is>
       </c>
       <c r="Q1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Cache write $/1M</t>
+          <t>Official Cache write $/1M</t>
         </is>
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI Output $/1M</t>
+          <t>Official Output $/1M</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
@@ -10368,7 +11456,7 @@
       </c>
       <c r="T1" s="2" t="inlineStr">
         <is>
-          <t>OpenAI note</t>
+          <t>Official note</t>
         </is>
       </c>
     </row>
@@ -18057,7 +19145,14 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Green columns: official OpenAI prices from https://developers.openai.com/api/docs/pricing (Standard tier; Batch tier for ':batch' models). Yellow rows: models OpenRouter does not list.</t>
+          <t>Green columns (OpenAI): official prices from https://developers.openai.com/api/docs/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
         </is>
       </c>
     </row>
@@ -18073,7 +19168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:T41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18088,6 +19183,14 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18151,6 +19254,46 @@
           <t>Web search $</t>
         </is>
       </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Official model</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Official tier</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Official Input $/1M</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cached input $/1M</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cache write $/1M</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Official Output $/1M</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Official note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18189,6 +19332,38 @@
       <c r="L2" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>claude-fable-5</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1h cache write: $20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18227,6 +19402,38 @@
       <c r="L3" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>claude-fable-5.1</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>1h cache write: $20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18265,6 +19472,29 @@
       <c r="L4" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>claude-fable-5.1</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18303,6 +19533,29 @@
       <c r="L5" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>claude-fable-5</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18341,6 +19594,38 @@
       <c r="L6" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>claude-haiku-4.5</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>1h cache write: $2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18379,6 +19664,29 @@
       <c r="L7" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>claude-haiku-4.5</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18417,6 +19725,38 @@
       <c r="L8" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>claude-opus-4.1</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>1h cache write: $30; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18455,6 +19795,34 @@
       <c r="L9" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>claude-opus-4.1</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18493,6 +19861,38 @@
       <c r="L10" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>claude-opus-4.5</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18531,6 +19931,29 @@
       <c r="L11" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>claude-opus-4.5</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P11" s="4" t="n"/>
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S11" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18569,6 +19992,38 @@
       <c r="L12" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>claude-opus-4.6</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -18607,6 +20062,29 @@
       <c r="L13" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>claude-opus-4.6</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P13" s="4" t="n"/>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -18645,6 +20123,38 @@
       <c r="L14" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>claude-opus-4.7</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -18683,6 +20193,29 @@
       <c r="L15" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>claude-opus-4.7</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P15" s="4" t="n"/>
+      <c r="Q15" s="4" t="n"/>
+      <c r="R15" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -18721,6 +20254,38 @@
       <c r="L16" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>claude-opus-4.8</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -18759,6 +20324,29 @@
       <c r="L17" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>claude-opus-4.8</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n"/>
+      <c r="R17" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -18797,6 +20385,38 @@
       <c r="L18" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>claude-opus-5</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="R18" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>1h cache write: $10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -18835,6 +20455,38 @@
       <c r="L19" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>claude-opus-5.5</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1h cache write: $8</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -18873,6 +20525,29 @@
       <c r="L20" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>claude-opus-5.5</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -18911,6 +20586,29 @@
       <c r="L21" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>claude-opus-5</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="n"/>
+      <c r="R21" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -18949,6 +20647,38 @@
       <c r="L22" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>1h cache write: $6; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18987,6 +20717,38 @@
       <c r="L23" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.5</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P23" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>1h cache write: $6</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -19025,6 +20787,29 @@
       <c r="L24" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.5</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -19063,6 +20848,38 @@
       <c r="L25" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.6</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P25" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q25" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>1h cache write: $6</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -19101,6 +20918,29 @@
       <c r="L26" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4.6</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -19139,6 +20979,38 @@
       <c r="L27" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P27" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q27" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="R27" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>1h cache write: $4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -19177,16 +21049,483 @@
       <c r="L28" s="4" t="n">
         <v>0.01</v>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>claude-sonnet-5</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" s="4" t="n"/>
+      <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S28" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9" t="n"/>
+      <c r="L29" s="9" t="n"/>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>claude-haiku-3.5</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O29" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="P29" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q29" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R29" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S29" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $1.6; retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" s="9" t="n"/>
+      <c r="J30" s="9" t="n"/>
+      <c r="K30" s="9" t="n"/>
+      <c r="L30" s="9" t="n"/>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5</t>
+        </is>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O30" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R30" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="S30" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $20; limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="9" t="n"/>
+      <c r="L31" s="9" t="n"/>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5.1</t>
+        </is>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O31" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="P31" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Q31" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="R31" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="S31" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $20; limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" s="9" t="n"/>
+      <c r="J32" s="9" t="n"/>
+      <c r="K32" s="9" t="n"/>
+      <c r="L32" s="9" t="n"/>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>claude-opus-4</t>
+        </is>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O32" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="P32" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q32" s="9" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="R32" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="S32" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T32" s="7" t="inlineStr">
+        <is>
+          <t>1h cache write: $30; retired, except on Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" s="9" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9" t="n"/>
+      <c r="L33" s="9" t="n"/>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>claude-haiku-3.5</t>
+        </is>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O33" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P33" s="9" t="n"/>
+      <c r="Q33" s="9" t="n"/>
+      <c r="R33" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S33" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="9" t="n"/>
+      <c r="L34" s="9" t="n"/>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5</t>
+        </is>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O34" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P34" s="9" t="n"/>
+      <c r="Q34" s="9" t="n"/>
+      <c r="R34" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="S34" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T34" s="7" t="inlineStr">
+        <is>
+          <t>limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>claude-mythos-5.1</t>
+        </is>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O35" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P35" s="9" t="n"/>
+      <c r="Q35" s="9" t="n"/>
+      <c r="R35" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="S35" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>limited availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
+      <c r="L36" s="9" t="n"/>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>claude-opus-4</t>
+        </is>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O36" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P36" s="9" t="n"/>
+      <c r="Q36" s="9" t="n"/>
+      <c r="R36" s="9" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="S36" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T36" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>anthropic</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="9" t="n"/>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>claude-sonnet-4</t>
+        </is>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="O37" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P37" s="9" t="n"/>
+      <c r="Q37" s="9" t="n"/>
+      <c r="R37" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>Only on Anthropic</t>
+        </is>
+      </c>
+      <c r="T37" s="7" t="inlineStr">
+        <is>
+          <t>retired, except on Bedrock and Google Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Green columns (Anthropic): official prices from https://platform.claude.com/docs/en/about-claude/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L28"/>
+  <autoFilter ref="A1:T37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add official DeepSeek and Cohere prices next to OpenRouter prices
DeepSeek: parse the models & pricing table (peak price in the columns,
off-peak in the note). Cohere: parse the model cards embedded in the
pricing page plus the older models listed in its FAQ. Every sheet now
carries the official-price columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmrknBAh1G6gZXqySqNkyo
</commit_message>
<xml_diff>
--- a/openrouter_prices.xlsx
+++ b/openrouter_prices.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Cohere" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All'!$A$1:$T$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All'!$A$1:$T$216</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OpenAI'!$A$1:$T$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Anthropic'!$A$1:$T$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DeepSeek'!$A$1:$L$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cohere'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DeepSeek'!$A$1:$T$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cohere'!$A$1:$T$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T210"/>
+  <dimension ref="A1:T223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8022,6 +8022,11 @@
       <c r="P129" s="4" t="n"/>
       <c r="Q129" s="4" t="n"/>
       <c r="R129" s="4" t="n"/>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8058,6 +8063,11 @@
       <c r="P130" s="4" t="n"/>
       <c r="Q130" s="4" t="n"/>
       <c r="R130" s="4" t="n"/>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8096,6 +8106,11 @@
       <c r="P131" s="4" t="n"/>
       <c r="Q131" s="4" t="n"/>
       <c r="R131" s="4" t="n"/>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8132,6 +8147,11 @@
       <c r="P132" s="4" t="n"/>
       <c r="Q132" s="4" t="n"/>
       <c r="R132" s="4" t="n"/>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8170,6 +8190,11 @@
       <c r="P133" s="4" t="n"/>
       <c r="Q133" s="4" t="n"/>
       <c r="R133" s="4" t="n"/>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8206,6 +8231,11 @@
       <c r="P134" s="4" t="n"/>
       <c r="Q134" s="4" t="n"/>
       <c r="R134" s="4" t="n"/>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8244,6 +8274,11 @@
       <c r="P135" s="4" t="n"/>
       <c r="Q135" s="4" t="n"/>
       <c r="R135" s="4" t="n"/>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -8282,6 +8317,11 @@
       <c r="P136" s="4" t="n"/>
       <c r="Q136" s="4" t="n"/>
       <c r="R136" s="4" t="n"/>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -8318,6 +8358,11 @@
       <c r="P137" s="4" t="n"/>
       <c r="Q137" s="4" t="n"/>
       <c r="R137" s="4" t="n"/>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8352,10 +8397,36 @@
       <c r="J138" s="4" t="n"/>
       <c r="K138" s="4" t="n"/>
       <c r="L138" s="4" t="n"/>
-      <c r="O138" s="4" t="n"/>
-      <c r="P138" s="4" t="n"/>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O138" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P138" s="4" t="n">
+        <v>0.006</v>
+      </c>
       <c r="Q138" s="4" t="n"/>
-      <c r="R138" s="4" t="n"/>
+      <c r="R138" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S138" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>Matched as 'deepseek-v4.1-flash'; Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -8394,6 +8465,11 @@
       <c r="P139" s="4" t="n"/>
       <c r="Q139" s="4" t="n"/>
       <c r="R139" s="4" t="n"/>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -8428,10 +8504,36 @@
       <c r="J140" s="4" t="n"/>
       <c r="K140" s="4" t="n"/>
       <c r="L140" s="4" t="n"/>
-      <c r="O140" s="4" t="n"/>
-      <c r="P140" s="4" t="n"/>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O140" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P140" s="4" t="n">
+        <v>0.006</v>
+      </c>
       <c r="Q140" s="4" t="n"/>
-      <c r="R140" s="4" t="n"/>
+      <c r="R140" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S140" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>Matched as 'deepseek-v4.1-flash'; Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -8470,6 +8572,11 @@
       <c r="P141" s="4" t="n"/>
       <c r="Q141" s="4" t="n"/>
       <c r="R141" s="4" t="n"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -8504,10 +8611,36 @@
       <c r="J142" s="4" t="n"/>
       <c r="K142" s="4" t="n"/>
       <c r="L142" s="4" t="n"/>
-      <c r="O142" s="4" t="n"/>
-      <c r="P142" s="4" t="n"/>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro-0813</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O142" s="4" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="P142" s="4" t="n">
+        <v>0.044</v>
+      </c>
       <c r="Q142" s="4" t="n"/>
-      <c r="R142" s="4" t="n"/>
+      <c r="R142" s="4" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="S142" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Peak-hour price; off-peak (half): in 0.66 / cached 0.022 / out 1.98</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -8542,10 +8675,36 @@
       <c r="J143" s="4" t="n"/>
       <c r="K143" s="4" t="n"/>
       <c r="L143" s="4" t="n"/>
-      <c r="O143" s="4" t="n"/>
-      <c r="P143" s="4" t="n"/>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O143" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P143" s="4" t="n">
+        <v>0.006</v>
+      </c>
       <c r="Q143" s="4" t="n"/>
-      <c r="R143" s="4" t="n"/>
+      <c r="R143" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S143" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -8584,6 +8743,11 @@
       <c r="P144" s="4" t="n"/>
       <c r="Q144" s="4" t="n"/>
       <c r="R144" s="4" t="n"/>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -8620,6 +8784,11 @@
       <c r="P145" s="4" t="n"/>
       <c r="Q145" s="4" t="n"/>
       <c r="R145" s="4" t="n"/>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Not on Cohere page</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -8654,10 +8823,34 @@
       <c r="J146" s="4" t="n"/>
       <c r="K146" s="4" t="n"/>
       <c r="L146" s="4" t="n"/>
-      <c r="O146" s="4" t="n"/>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>command-a-plus</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O146" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="P146" s="4" t="n"/>
       <c r="Q146" s="4" t="n"/>
-      <c r="R146" s="4" t="n"/>
+      <c r="R146" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S146" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Free (open-weights model)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -8690,10 +8883,34 @@
       <c r="J147" s="4" t="n"/>
       <c r="K147" s="4" t="n"/>
       <c r="L147" s="4" t="n"/>
-      <c r="O147" s="4" t="n"/>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>command-r</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O147" s="4" t="n">
+        <v>0.15</v>
+      </c>
       <c r="P147" s="4" t="n"/>
       <c r="Q147" s="4" t="n"/>
-      <c r="R147" s="4" t="n"/>
+      <c r="R147" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S147" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Matched as 'command-r'</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -8726,10 +8943,34 @@
       <c r="J148" s="4" t="n"/>
       <c r="K148" s="4" t="n"/>
       <c r="L148" s="4" t="n"/>
-      <c r="O148" s="4" t="n"/>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>command-r-plus-08-2024</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O148" s="4" t="n">
+        <v>2.5</v>
+      </c>
       <c r="P148" s="4" t="n"/>
       <c r="Q148" s="4" t="n"/>
-      <c r="R148" s="4" t="n"/>
+      <c r="R148" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S148" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -8762,10 +9003,34 @@
       <c r="J149" s="4" t="n"/>
       <c r="K149" s="4" t="n"/>
       <c r="L149" s="4" t="n"/>
-      <c r="O149" s="4" t="n"/>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>command-r7b</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O149" s="4" t="n">
+        <v>0.0375</v>
+      </c>
       <c r="P149" s="4" t="n"/>
       <c r="Q149" s="4" t="n"/>
-      <c r="R149" s="4" t="n"/>
+      <c r="R149" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S149" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Matched as 'command-r7b'</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8798,10 +9063,34 @@
       <c r="J150" s="4" t="n"/>
       <c r="K150" s="4" t="n"/>
       <c r="L150" s="4" t="n"/>
-      <c r="O150" s="4" t="n"/>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>north-mini-code</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O150" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="P150" s="4" t="n"/>
       <c r="Q150" s="4" t="n"/>
-      <c r="R150" s="4" t="n"/>
+      <c r="R150" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S150" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Free (open-weights model)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11293,36 +11582,538 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B206" s="7" t="n"/>
+      <c r="C206" s="7" t="n"/>
+      <c r="D206" s="8" t="n"/>
+      <c r="E206" s="9" t="n"/>
+      <c r="F206" s="9" t="n"/>
+      <c r="G206" s="9" t="n"/>
+      <c r="H206" s="9" t="n"/>
+      <c r="I206" s="9" t="n"/>
+      <c r="J206" s="9" t="n"/>
+      <c r="K206" s="9" t="n"/>
+      <c r="L206" s="9" t="n"/>
+      <c r="M206" s="7" t="inlineStr">
+        <is>
+          <t>aya-expanse-32b</t>
+        </is>
+      </c>
+      <c r="N206" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O206" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P206" s="9" t="n"/>
+      <c r="Q206" s="9" t="n"/>
+      <c r="R206" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S206" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T206" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
     <row r="207">
-      <c r="A207" t="inlineStr">
+      <c r="A207" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B207" s="7" t="n"/>
+      <c r="C207" s="7" t="n"/>
+      <c r="D207" s="8" t="n"/>
+      <c r="E207" s="9" t="n"/>
+      <c r="F207" s="9" t="n"/>
+      <c r="G207" s="9" t="n"/>
+      <c r="H207" s="9" t="n"/>
+      <c r="I207" s="9" t="n"/>
+      <c r="J207" s="9" t="n"/>
+      <c r="K207" s="9" t="n"/>
+      <c r="L207" s="9" t="n"/>
+      <c r="M207" s="7" t="inlineStr">
+        <is>
+          <t>aya-expanse-8b</t>
+        </is>
+      </c>
+      <c r="N207" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O207" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P207" s="9" t="n"/>
+      <c r="Q207" s="9" t="n"/>
+      <c r="R207" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S207" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T207" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B208" s="7" t="n"/>
+      <c r="C208" s="7" t="n"/>
+      <c r="D208" s="8" t="n"/>
+      <c r="E208" s="9" t="n"/>
+      <c r="F208" s="9" t="n"/>
+      <c r="G208" s="9" t="n"/>
+      <c r="H208" s="9" t="n"/>
+      <c r="I208" s="9" t="n"/>
+      <c r="J208" s="9" t="n"/>
+      <c r="K208" s="9" t="n"/>
+      <c r="L208" s="9" t="n"/>
+      <c r="M208" s="7" t="inlineStr">
+        <is>
+          <t>command</t>
+        </is>
+      </c>
+      <c r="N208" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O208" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P208" s="9" t="n"/>
+      <c r="Q208" s="9" t="n"/>
+      <c r="R208" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S208" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T208" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B209" s="7" t="n"/>
+      <c r="C209" s="7" t="n"/>
+      <c r="D209" s="8" t="n"/>
+      <c r="E209" s="9" t="n"/>
+      <c r="F209" s="9" t="n"/>
+      <c r="G209" s="9" t="n"/>
+      <c r="H209" s="9" t="n"/>
+      <c r="I209" s="9" t="n"/>
+      <c r="J209" s="9" t="n"/>
+      <c r="K209" s="9" t="n"/>
+      <c r="L209" s="9" t="n"/>
+      <c r="M209" s="7" t="inlineStr">
+        <is>
+          <t>command-light</t>
+        </is>
+      </c>
+      <c r="N209" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O209" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P209" s="9" t="n"/>
+      <c r="Q209" s="9" t="n"/>
+      <c r="R209" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S209" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T209" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B210" s="7" t="n"/>
+      <c r="C210" s="7" t="n"/>
+      <c r="D210" s="8" t="n"/>
+      <c r="E210" s="9" t="n"/>
+      <c r="F210" s="9" t="n"/>
+      <c r="G210" s="9" t="n"/>
+      <c r="H210" s="9" t="n"/>
+      <c r="I210" s="9" t="n"/>
+      <c r="J210" s="9" t="n"/>
+      <c r="K210" s="9" t="n"/>
+      <c r="L210" s="9" t="n"/>
+      <c r="M210" s="7" t="inlineStr">
+        <is>
+          <t>command-r-03-2024</t>
+        </is>
+      </c>
+      <c r="N210" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O210" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P210" s="9" t="n"/>
+      <c r="Q210" s="9" t="n"/>
+      <c r="R210" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S210" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T210" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B211" s="7" t="n"/>
+      <c r="C211" s="7" t="n"/>
+      <c r="D211" s="8" t="n"/>
+      <c r="E211" s="9" t="n"/>
+      <c r="F211" s="9" t="n"/>
+      <c r="G211" s="9" t="n"/>
+      <c r="H211" s="9" t="n"/>
+      <c r="I211" s="9" t="n"/>
+      <c r="J211" s="9" t="n"/>
+      <c r="K211" s="9" t="n"/>
+      <c r="L211" s="9" t="n"/>
+      <c r="M211" s="7" t="inlineStr">
+        <is>
+          <t>command-r-plus-04-2024</t>
+        </is>
+      </c>
+      <c r="N211" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O211" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P211" s="9" t="n"/>
+      <c r="Q211" s="9" t="n"/>
+      <c r="R211" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="S211" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T211" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B212" s="7" t="n"/>
+      <c r="C212" s="7" t="n"/>
+      <c r="D212" s="8" t="n"/>
+      <c r="E212" s="9" t="n"/>
+      <c r="F212" s="9" t="n"/>
+      <c r="G212" s="9" t="n"/>
+      <c r="H212" s="9" t="n"/>
+      <c r="I212" s="9" t="n"/>
+      <c r="J212" s="9" t="n"/>
+      <c r="K212" s="9" t="n"/>
+      <c r="L212" s="9" t="n"/>
+      <c r="M212" s="7" t="inlineStr">
+        <is>
+          <t>embed-4</t>
+        </is>
+      </c>
+      <c r="N212" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O212" s="9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P212" s="9" t="n"/>
+      <c r="Q212" s="9" t="n"/>
+      <c r="R212" s="9" t="n"/>
+      <c r="S212" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T212" s="7" t="inlineStr">
+        <is>
+          <t>Image cost: $0.47 / 1M tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B213" s="7" t="n"/>
+      <c r="C213" s="7" t="n"/>
+      <c r="D213" s="8" t="n"/>
+      <c r="E213" s="9" t="n"/>
+      <c r="F213" s="9" t="n"/>
+      <c r="G213" s="9" t="n"/>
+      <c r="H213" s="9" t="n"/>
+      <c r="I213" s="9" t="n"/>
+      <c r="J213" s="9" t="n"/>
+      <c r="K213" s="9" t="n"/>
+      <c r="L213" s="9" t="n"/>
+      <c r="M213" s="7" t="inlineStr">
+        <is>
+          <t>parse-5</t>
+        </is>
+      </c>
+      <c r="N213" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O213" s="9" t="n"/>
+      <c r="P213" s="9" t="n"/>
+      <c r="Q213" s="9" t="n"/>
+      <c r="R213" s="9" t="n"/>
+      <c r="S213" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T213" s="7" t="inlineStr">
+        <is>
+          <t>$1.5 / 1K pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B214" s="7" t="n"/>
+      <c r="C214" s="7" t="n"/>
+      <c r="D214" s="8" t="n"/>
+      <c r="E214" s="9" t="n"/>
+      <c r="F214" s="9" t="n"/>
+      <c r="G214" s="9" t="n"/>
+      <c r="H214" s="9" t="n"/>
+      <c r="I214" s="9" t="n"/>
+      <c r="J214" s="9" t="n"/>
+      <c r="K214" s="9" t="n"/>
+      <c r="L214" s="9" t="n"/>
+      <c r="M214" s="7" t="inlineStr">
+        <is>
+          <t>rerank-4-fast</t>
+        </is>
+      </c>
+      <c r="N214" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O214" s="9" t="n"/>
+      <c r="P214" s="9" t="n"/>
+      <c r="Q214" s="9" t="n"/>
+      <c r="R214" s="9" t="n"/>
+      <c r="S214" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T214" s="7" t="inlineStr">
+        <is>
+          <t>$2 / 1K searches</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B215" s="7" t="n"/>
+      <c r="C215" s="7" t="n"/>
+      <c r="D215" s="8" t="n"/>
+      <c r="E215" s="9" t="n"/>
+      <c r="F215" s="9" t="n"/>
+      <c r="G215" s="9" t="n"/>
+      <c r="H215" s="9" t="n"/>
+      <c r="I215" s="9" t="n"/>
+      <c r="J215" s="9" t="n"/>
+      <c r="K215" s="9" t="n"/>
+      <c r="L215" s="9" t="n"/>
+      <c r="M215" s="7" t="inlineStr">
+        <is>
+          <t>rerank-4-pro</t>
+        </is>
+      </c>
+      <c r="N215" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O215" s="9" t="n"/>
+      <c r="P215" s="9" t="n"/>
+      <c r="Q215" s="9" t="n"/>
+      <c r="R215" s="9" t="n"/>
+      <c r="S215" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T215" s="7" t="inlineStr">
+        <is>
+          <t>$2.5 / 1K searches</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B216" s="7" t="n"/>
+      <c r="C216" s="7" t="n"/>
+      <c r="D216" s="8" t="n"/>
+      <c r="E216" s="9" t="n"/>
+      <c r="F216" s="9" t="n"/>
+      <c r="G216" s="9" t="n"/>
+      <c r="H216" s="9" t="n"/>
+      <c r="I216" s="9" t="n"/>
+      <c r="J216" s="9" t="n"/>
+      <c r="K216" s="9" t="n"/>
+      <c r="L216" s="9" t="n"/>
+      <c r="M216" s="7" t="inlineStr">
+        <is>
+          <t>transcribe</t>
+        </is>
+      </c>
+      <c r="N216" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O216" s="9" t="n"/>
+      <c r="P216" s="9" t="n"/>
+      <c r="Q216" s="9" t="n"/>
+      <c r="R216" s="9" t="n"/>
+      <c r="S216" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T216" s="7" t="inlineStr">
+        <is>
+          <t>$3.75 / hour / instance (via Model Vault)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
         <is>
           <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
         </is>
       </c>
     </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
+    <row r="219">
+      <c r="A219" t="inlineStr">
         <is>
           <t>Green columns (OpenAI): official prices from https://developers.openai.com/api/docs/pricing</t>
         </is>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
+    <row r="220">
+      <c r="A220" t="inlineStr">
         <is>
           <t>Green columns (Anthropic): official prices from https://platform.claude.com/docs/en/about-claude/pricing</t>
         </is>
       </c>
     </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Green columns (DeepSeek): official prices from https://api-docs.deepseek.com/quick_start/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Green columns (Cohere): official prices from https://cohere.com/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
         <is>
           <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T205"/>
+  <autoFilter ref="A1:T216"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21536,7 +22327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21551,6 +22342,14 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21612,6 +22411,46 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Web search $</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Official model</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Official tier</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Official Input $/1M</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cached input $/1M</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cache write $/1M</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Official Output $/1M</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Official note</t>
         </is>
       </c>
     </row>
@@ -21646,6 +22485,15 @@
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -21678,6 +22526,15 @@
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -21712,6 +22569,15 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -21744,6 +22610,15 @@
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -21778,6 +22653,15 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -21810,6 +22694,15 @@
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -21844,6 +22737,15 @@
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -21878,6 +22780,15 @@
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -21910,6 +22821,15 @@
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -21944,6 +22864,36 @@
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="n"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S11" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Matched as 'deepseek-v4.1-flash'; Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -21978,6 +22928,15 @@
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="4" t="n"/>
+      <c r="O12" s="4" t="n"/>
+      <c r="P12" s="4" t="n"/>
+      <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -22012,6 +22971,36 @@
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P13" s="4" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Matched as 'deepseek-v4.1-flash'; Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -22046,6 +23035,15 @@
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="4" t="n"/>
+      <c r="O14" s="4" t="n"/>
+      <c r="P14" s="4" t="n"/>
+      <c r="Q14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -22080,6 +23078,36 @@
       <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="n"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>deepseek-v4-pro-0813</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="P15" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="Q15" s="4" t="n"/>
+      <c r="R15" s="4" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="S15" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Peak-hour price; off-peak (half): in 0.66 / cached 0.022 / out 1.98</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -22114,6 +23142,36 @@
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="n"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>deepseek-v4.1-flash</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="Q16" s="4" t="n"/>
+      <c r="R16" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Peak-hour price; off-peak (half): in 0.15 / cached 0.003 / out 0.6</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -22148,6 +23206,15 @@
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Not on DeepSeek page</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -22156,8 +23223,22 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Green columns (DeepSeek): official prices from https://api-docs.deepseek.com/quick_start/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L17"/>
+  <autoFilter ref="A1:T17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22168,7 +23249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -22183,6 +23264,14 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22244,6 +23333,46 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Web search $</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Official model</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Official tier</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Official Input $/1M</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cached input $/1M</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Official Cache write $/1M</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Official Output $/1M</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Compare</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Official note</t>
         </is>
       </c>
     </row>
@@ -22278,6 +23407,15 @@
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
       <c r="L2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Not on Cohere page</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -22312,6 +23450,34 @@
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="n"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>command-a-plus</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Free (open-weights model)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -22344,6 +23510,34 @@
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>command-r</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Matched as 'command-r'</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -22376,6 +23570,34 @@
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>command-r-plus-08-2024</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -22408,6 +23630,34 @@
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>command-r7b</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Matched as 'command-r7b'</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -22440,16 +23690,546 @@
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>north-mini-code</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>Same</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Free (open-weights model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>aya-expanse-32b</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P8" s="9" t="n"/>
+      <c r="Q8" s="9" t="n"/>
+      <c r="R8" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>aya-expanse-8b</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P9" s="9" t="n"/>
+      <c r="Q9" s="9" t="n"/>
+      <c r="R9" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>command</t>
+        </is>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="9" t="n"/>
+      <c r="Q10" s="9" t="n"/>
+      <c r="R10" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>command-light</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>command-r-03-2024</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P12" s="9" t="n"/>
+      <c r="Q12" s="9" t="n"/>
+      <c r="R12" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9" t="n"/>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9" t="n"/>
+      <c r="L13" s="9" t="n"/>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>command-r-plus-04-2024</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" s="9" t="n"/>
+      <c r="Q13" s="9" t="n"/>
+      <c r="R13" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Listed in Cohere pricing FAQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="9" t="n"/>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>embed-4</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O14" s="9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P14" s="9" t="n"/>
+      <c r="Q14" s="9" t="n"/>
+      <c r="R14" s="9" t="n"/>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>Image cost: $0.47 / 1M tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="9" t="n"/>
+      <c r="L15" s="9" t="n"/>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>parse-5</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="n"/>
+      <c r="P15" s="9" t="n"/>
+      <c r="Q15" s="9" t="n"/>
+      <c r="R15" s="9" t="n"/>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>$1.5 / 1K pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>rerank-4-fast</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="n"/>
+      <c r="P16" s="9" t="n"/>
+      <c r="Q16" s="9" t="n"/>
+      <c r="R16" s="9" t="n"/>
+      <c r="S16" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>$2 / 1K searches</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>rerank-4-pro</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="n"/>
+      <c r="P17" s="9" t="n"/>
+      <c r="Q17" s="9" t="n"/>
+      <c r="R17" s="9" t="n"/>
+      <c r="S17" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>$2.5 / 1K searches</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>cohere</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="9" t="n"/>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="9" t="n"/>
+      <c r="L18" s="9" t="n"/>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>transcribe</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="n"/>
+      <c r="P18" s="9" t="n"/>
+      <c r="Q18" s="9" t="n"/>
+      <c r="R18" s="9" t="n"/>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
+          <t>Only on Cohere</t>
+        </is>
+      </c>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>$3.75 / hour / instance (via Model Vault)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Green columns (Cohere): official prices from https://cohere.com/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Standard tier, or Batch tier for ':batch' models. Yellow rows: models OpenRouter does not list.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:T18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use each model's openrouter.ai page price and flag deprecated models
OpenRouter prices now come from the price shown on each model's page
(input, output and cache prices from its FAQ), which is the cheapest
active provider, instead of the models API default. When a page shows
no price the model is treated as removed from OpenRouter, unless the API
still lists it.

The comparison and offer lists gain availability columns: removed from
OpenRouter, scheduled for removal (API expiration_date), retired by the
maker, or missing from the maker's pricing page, shaded grey by how
certain the deprecation is.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmrknBAh1G6gZXqySqNkyo
</commit_message>
<xml_diff>
--- a/openrouter_prices.xlsx
+++ b/openrouter_prices.xlsx
@@ -1218,7 +1218,7 @@
         <v>0.4</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
@@ -1247,9 +1247,9 @@
       <c r="R13" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -1396,9 +1396,7 @@
       <c r="F16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G16" s="4" t="n">
-        <v>1.25</v>
-      </c>
+      <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -1968,7 +1966,7 @@
         <v>2</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -1997,9 +1995,9 @@
       <c r="R27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="S27" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2088,7 @@
         <v>0.4</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
@@ -2119,9 +2117,9 @@
       <c r="R29" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="S29" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S29" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2324,7 @@
         <v>10</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.125</v>
+        <v>0.13</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -2355,9 +2353,9 @@
       <c r="R33" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="S33" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S33" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -5353,13 +5351,13 @@
         <v>131072</v>
       </c>
       <c r="E86" s="4" t="n">
-        <v>0.15</v>
+        <v>0.03</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>0.6</v>
+        <v>0.17</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>0.075</v>
+        <v>0.03</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -8010,7 +8008,7 @@
         <v>0.2574</v>
       </c>
       <c r="F129" s="4" t="n">
-        <v>1.0287</v>
+        <v>1.029</v>
       </c>
       <c r="G129" s="4" t="n"/>
       <c r="H129" s="4" t="n"/>
@@ -8048,12 +8046,14 @@
         <v>163840</v>
       </c>
       <c r="E130" s="4" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F130" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G130" s="4" t="n"/>
+        <v>0.9</v>
+      </c>
+      <c r="G130" s="4" t="n">
+        <v>0.135</v>
+      </c>
       <c r="H130" s="4" t="n"/>
       <c r="I130" s="4" t="n"/>
       <c r="J130" s="4" t="n"/>
@@ -8262,9 +8262,7 @@
       <c r="F135" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G135" s="4" t="n">
-        <v>0.135</v>
-      </c>
+      <c r="G135" s="4" t="n"/>
       <c r="H135" s="4" t="n"/>
       <c r="I135" s="4" t="n"/>
       <c r="J135" s="4" t="n"/>
@@ -8300,13 +8298,13 @@
         <v>163840</v>
       </c>
       <c r="E136" s="4" t="n">
-        <v>0.269</v>
+        <v>0.2088</v>
       </c>
       <c r="F136" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3096</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>0.1345</v>
+        <v>0.0216</v>
       </c>
       <c r="H136" s="4" t="n"/>
       <c r="I136" s="4" t="n"/>
@@ -8384,13 +8382,13 @@
         <v>1048576</v>
       </c>
       <c r="E138" s="4" t="n">
-        <v>0.0469</v>
+        <v>0.03</v>
       </c>
       <c r="F138" s="4" t="n">
-        <v>0.09379999999999999</v>
+        <v>1.28</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>0.0094</v>
+        <v>0.016</v>
       </c>
       <c r="H138" s="4" t="n"/>
       <c r="I138" s="4" t="n"/>
@@ -8555,13 +8553,13 @@
         <v>1048576</v>
       </c>
       <c r="E141" s="4" t="n">
-        <v>0.348</v>
+        <v>0.9553</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>0.696</v>
+        <v>1.911</v>
       </c>
       <c r="G141" s="4" t="n">
-        <v>0.029</v>
+        <v>0.0796</v>
       </c>
       <c r="H141" s="4" t="n"/>
       <c r="I141" s="4" t="n"/>
@@ -8598,13 +8596,13 @@
         <v>1048576</v>
       </c>
       <c r="E142" s="4" t="n">
-        <v>0.245</v>
+        <v>0.128</v>
       </c>
       <c r="F142" s="4" t="n">
-        <v>3.5</v>
+        <v>1.958</v>
       </c>
       <c r="G142" s="4" t="n">
-        <v>0.2445</v>
+        <v>0.0883</v>
       </c>
       <c r="H142" s="4" t="n"/>
       <c r="I142" s="4" t="n"/>
@@ -8662,13 +8660,13 @@
         <v>1048576</v>
       </c>
       <c r="E143" s="4" t="n">
-        <v>0.035</v>
+        <v>0.02</v>
       </c>
       <c r="F143" s="4" t="n">
-        <v>0.29</v>
+        <v>0.6</v>
       </c>
       <c r="G143" s="4" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="H143" s="4" t="n"/>
       <c r="I143" s="4" t="n"/>
@@ -12073,7 +12071,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
+          <t>Source: each model's page on openrouter.ai (In / Out Price), fetched 2026-09-28. Empty = not applicable.</t>
         </is>
       </c>
     </row>
@@ -12875,7 +12873,7 @@
         <v>0.4</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
@@ -12904,9 +12902,9 @@
       <c r="R13" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S13" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -13053,9 +13051,7 @@
       <c r="F16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G16" s="4" t="n">
-        <v>1.25</v>
-      </c>
+      <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
@@ -13625,7 +13621,7 @@
         <v>2</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
@@ -13654,9 +13650,9 @@
       <c r="R27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="S27" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -13747,7 +13743,7 @@
         <v>0.4</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
@@ -13776,9 +13772,9 @@
       <c r="R29" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="S29" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S29" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -13983,7 +13979,7 @@
         <v>10</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.125</v>
+        <v>0.13</v>
       </c>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
@@ -14012,9 +14008,9 @@
       <c r="R33" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="S33" s="5" t="inlineStr">
-        <is>
-          <t>Same</t>
+      <c r="S33" s="6" t="inlineStr">
+        <is>
+          <t>Different</t>
         </is>
       </c>
     </row>
@@ -17010,13 +17006,13 @@
         <v>131072</v>
       </c>
       <c r="E86" s="4" t="n">
-        <v>0.15</v>
+        <v>0.03</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>0.6</v>
+        <v>0.17</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>0.075</v>
+        <v>0.03</v>
       </c>
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
@@ -19929,7 +19925,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
+          <t>Source: each model's page on openrouter.ai (In / Out Price), fetched 2026-09-28. Empty = not applicable.</t>
         </is>
       </c>
     </row>
@@ -22297,7 +22293,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
+          <t>Source: each model's page on openrouter.ai (In / Out Price), fetched 2026-09-28. Empty = not applicable.</t>
         </is>
       </c>
     </row>
@@ -22477,7 +22473,7 @@
         <v>0.2574</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.0287</v>
+        <v>1.029</v>
       </c>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
@@ -22515,12 +22511,14 @@
         <v>163840</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4" t="n"/>
+        <v>0.9</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0.135</v>
+      </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
@@ -22729,9 +22727,7 @@
       <c r="F8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="4" t="n">
-        <v>0.135</v>
-      </c>
+      <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
@@ -22767,13 +22763,13 @@
         <v>163840</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.269</v>
+        <v>0.2088</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.4</v>
+        <v>0.3096</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.1345</v>
+        <v>0.0216</v>
       </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
@@ -22851,13 +22847,13 @@
         <v>1048576</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.0469</v>
+        <v>0.03</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.09379999999999999</v>
+        <v>1.28</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.0094</v>
+        <v>0.016</v>
       </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
@@ -23022,13 +23018,13 @@
         <v>1048576</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.348</v>
+        <v>0.9553</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.696</v>
+        <v>1.911</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.029</v>
+        <v>0.0796</v>
       </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
@@ -23065,13 +23061,13 @@
         <v>1048576</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.245</v>
+        <v>0.128</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>3.5</v>
+        <v>1.958</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.2445</v>
+        <v>0.0883</v>
       </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
@@ -23129,13 +23125,13 @@
         <v>1048576</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.035</v>
+        <v>0.02</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.29</v>
+        <v>0.6</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
@@ -23219,7 +23215,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
+          <t>Source: each model's page on openrouter.ai (In / Out Price), fetched 2026-09-28. Empty = not applicable.</t>
         </is>
       </c>
     </row>
@@ -24210,7 +24206,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Source: https://openrouter.ai/api/v1/models — fetched 2026-09-27. Empty = not applicable.</t>
+          <t>Source: each model's page on openrouter.ai (In / Out Price), fetched 2026-09-28. Empty = not applicable.</t>
         </is>
       </c>
     </row>

</xml_diff>